<commit_message>
Revise printe view template
</commit_message>
<xml_diff>
--- a/templates/Spec.xlsx
+++ b/templates/Spec.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IT06-PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\QC Web App\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976C6621-49BA-4C67-9E16-F90ECFB4D408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DEC55E6-9B5F-4BFC-B2CE-B9050C78361E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spec" sheetId="16" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="74">
   <si>
     <t>MARUNIX(CAMBODIA)Co.,Ltd</t>
   </si>
@@ -278,21 +278,6 @@
   <si>
     <t>អ្នកត្រួតពិនិត្យ
 [Inspector]</t>
-  </si>
-  <si>
-    <t>REF:  QC-RE-002   REV:03   Date: 02/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> តារាងត្រួតពិនិត្យផលិតផល
-[OQC Inspection record]</t>
-  </si>
-  <si>
-    <t>សំរេចជារួម
-[Total Determination]</t>
-  </si>
-  <si>
-    <t>ត្រួតពិនិ្យដោយ
-[Checked by]</t>
   </si>
 </sst>
 </file>
@@ -1415,6 +1400,270 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1450,270 +1699,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1742,14 +1727,20 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Wire"/>
+        <xdr:cNvPr id="2" name="Wire">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1799,14 +1790,20 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Terminal"/>
+        <xdr:cNvPr id="3" name="Terminal">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1856,14 +1853,20 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Housing"/>
+        <xdr:cNvPr id="4" name="Housing">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1913,14 +1916,20 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Other"/>
+        <xdr:cNvPr id="5" name="Other">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2324,7 +2333,7 @@
     <col min="6" max="6" width="3.125" style="5" customWidth="1"/>
     <col min="7" max="7" width="1.75" style="5" customWidth="1"/>
     <col min="8" max="8" width="2.25" style="5" customWidth="1"/>
-    <col min="9" max="9" width="4.625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="5" style="5" customWidth="1"/>
     <col min="10" max="10" width="2.5" style="5" customWidth="1"/>
     <col min="11" max="12" width="3.625" style="5" customWidth="1"/>
     <col min="13" max="15" width="2" style="5" customWidth="1"/>
@@ -2419,33 +2428,33 @@
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
       <c r="N2" s="6"/>
-      <c r="O2" s="86" t="s">
+      <c r="O2" s="174" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="86"/>
-      <c r="Q2" s="86"/>
-      <c r="R2" s="86"/>
-      <c r="S2" s="86"/>
-      <c r="T2" s="86"/>
-      <c r="U2" s="86"/>
-      <c r="V2" s="86"/>
-      <c r="W2" s="86"/>
-      <c r="X2" s="86"/>
-      <c r="Y2" s="86"/>
-      <c r="Z2" s="86"/>
-      <c r="AA2" s="86"/>
-      <c r="AB2" s="86"/>
-      <c r="AC2" s="86"/>
-      <c r="AD2" s="86"/>
-      <c r="AE2" s="86"/>
-      <c r="AF2" s="86"/>
-      <c r="AG2" s="86"/>
-      <c r="AH2" s="86"/>
-      <c r="AI2" s="86"/>
-      <c r="AJ2" s="86"/>
-      <c r="AK2" s="86"/>
-      <c r="AL2" s="86"/>
-      <c r="AM2" s="86"/>
+      <c r="P2" s="174"/>
+      <c r="Q2" s="174"/>
+      <c r="R2" s="174"/>
+      <c r="S2" s="174"/>
+      <c r="T2" s="174"/>
+      <c r="U2" s="174"/>
+      <c r="V2" s="174"/>
+      <c r="W2" s="174"/>
+      <c r="X2" s="174"/>
+      <c r="Y2" s="174"/>
+      <c r="Z2" s="174"/>
+      <c r="AA2" s="174"/>
+      <c r="AB2" s="174"/>
+      <c r="AC2" s="174"/>
+      <c r="AD2" s="174"/>
+      <c r="AE2" s="174"/>
+      <c r="AF2" s="174"/>
+      <c r="AG2" s="174"/>
+      <c r="AH2" s="174"/>
+      <c r="AI2" s="174"/>
+      <c r="AJ2" s="174"/>
+      <c r="AK2" s="174"/>
+      <c r="AL2" s="174"/>
+      <c r="AM2" s="174"/>
     </row>
     <row r="3" spans="1:50" ht="29.25" customHeight="1">
       <c r="B3" s="9"/>
@@ -2461,38 +2470,38 @@
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="6"/>
-      <c r="O3" s="86"/>
-      <c r="P3" s="86"/>
-      <c r="Q3" s="86"/>
-      <c r="R3" s="86"/>
-      <c r="S3" s="86"/>
-      <c r="T3" s="86"/>
-      <c r="U3" s="86"/>
-      <c r="V3" s="86"/>
-      <c r="W3" s="86"/>
-      <c r="X3" s="86"/>
-      <c r="Y3" s="86"/>
-      <c r="Z3" s="86"/>
-      <c r="AA3" s="86"/>
-      <c r="AB3" s="86"/>
-      <c r="AC3" s="86"/>
-      <c r="AD3" s="86"/>
-      <c r="AE3" s="86"/>
-      <c r="AF3" s="86"/>
-      <c r="AG3" s="86"/>
-      <c r="AH3" s="86"/>
-      <c r="AI3" s="86"/>
-      <c r="AJ3" s="86"/>
-      <c r="AK3" s="86"/>
-      <c r="AL3" s="86"/>
-      <c r="AM3" s="86"/>
-      <c r="AO3" s="87" t="s">
+      <c r="O3" s="174"/>
+      <c r="P3" s="174"/>
+      <c r="Q3" s="174"/>
+      <c r="R3" s="174"/>
+      <c r="S3" s="174"/>
+      <c r="T3" s="174"/>
+      <c r="U3" s="174"/>
+      <c r="V3" s="174"/>
+      <c r="W3" s="174"/>
+      <c r="X3" s="174"/>
+      <c r="Y3" s="174"/>
+      <c r="Z3" s="174"/>
+      <c r="AA3" s="174"/>
+      <c r="AB3" s="174"/>
+      <c r="AC3" s="174"/>
+      <c r="AD3" s="174"/>
+      <c r="AE3" s="174"/>
+      <c r="AF3" s="174"/>
+      <c r="AG3" s="174"/>
+      <c r="AH3" s="174"/>
+      <c r="AI3" s="174"/>
+      <c r="AJ3" s="174"/>
+      <c r="AK3" s="174"/>
+      <c r="AL3" s="174"/>
+      <c r="AM3" s="174"/>
+      <c r="AO3" s="175" t="s">
         <v>4</v>
       </c>
-      <c r="AP3" s="87"/>
-      <c r="AQ3" s="87"/>
-      <c r="AR3" s="87"/>
-      <c r="AS3" s="87"/>
+      <c r="AP3" s="175"/>
+      <c r="AQ3" s="175"/>
+      <c r="AR3" s="175"/>
+      <c r="AS3" s="175"/>
       <c r="AU3" s="10"/>
       <c r="AV3" s="10"/>
     </row>
@@ -2538,178 +2547,178 @@
       <c r="AO4" s="9"/>
     </row>
     <row r="5" spans="1:50" s="13" customFormat="1" ht="27" customHeight="1">
-      <c r="A5" s="88" t="s">
+      <c r="A5" s="176" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="89"/>
-      <c r="C5" s="89"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="89"/>
-      <c r="F5" s="89"/>
-      <c r="G5" s="89"/>
-      <c r="H5" s="90"/>
-      <c r="I5" s="91" t="s">
+      <c r="B5" s="177"/>
+      <c r="C5" s="177"/>
+      <c r="D5" s="177"/>
+      <c r="E5" s="177"/>
+      <c r="F5" s="177"/>
+      <c r="G5" s="177"/>
+      <c r="H5" s="178"/>
+      <c r="I5" s="179" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="89"/>
-      <c r="K5" s="89"/>
-      <c r="L5" s="89"/>
-      <c r="M5" s="89"/>
-      <c r="N5" s="89"/>
-      <c r="O5" s="89"/>
-      <c r="P5" s="89"/>
-      <c r="Q5" s="89"/>
-      <c r="R5" s="89"/>
-      <c r="S5" s="89"/>
-      <c r="T5" s="89"/>
-      <c r="U5" s="91" t="s">
+      <c r="J5" s="177"/>
+      <c r="K5" s="177"/>
+      <c r="L5" s="177"/>
+      <c r="M5" s="177"/>
+      <c r="N5" s="177"/>
+      <c r="O5" s="177"/>
+      <c r="P5" s="177"/>
+      <c r="Q5" s="177"/>
+      <c r="R5" s="177"/>
+      <c r="S5" s="177"/>
+      <c r="T5" s="177"/>
+      <c r="U5" s="179" t="s">
         <v>7</v>
       </c>
-      <c r="V5" s="89"/>
-      <c r="W5" s="89"/>
-      <c r="X5" s="89"/>
-      <c r="Y5" s="89"/>
-      <c r="Z5" s="89"/>
-      <c r="AA5" s="90"/>
-      <c r="AB5" s="91" t="s">
+      <c r="V5" s="177"/>
+      <c r="W5" s="177"/>
+      <c r="X5" s="177"/>
+      <c r="Y5" s="177"/>
+      <c r="Z5" s="177"/>
+      <c r="AA5" s="178"/>
+      <c r="AB5" s="179" t="s">
         <v>8</v>
       </c>
-      <c r="AC5" s="89"/>
-      <c r="AD5" s="89"/>
-      <c r="AE5" s="89"/>
-      <c r="AF5" s="89"/>
-      <c r="AG5" s="89"/>
-      <c r="AH5" s="90"/>
-      <c r="AI5" s="91" t="s">
+      <c r="AC5" s="177"/>
+      <c r="AD5" s="177"/>
+      <c r="AE5" s="177"/>
+      <c r="AF5" s="177"/>
+      <c r="AG5" s="177"/>
+      <c r="AH5" s="178"/>
+      <c r="AI5" s="179" t="s">
         <v>9</v>
       </c>
-      <c r="AJ5" s="89"/>
-      <c r="AK5" s="89"/>
-      <c r="AL5" s="89"/>
-      <c r="AM5" s="89"/>
-      <c r="AN5" s="89"/>
-      <c r="AO5" s="89"/>
-      <c r="AP5" s="91" t="s">
+      <c r="AJ5" s="177"/>
+      <c r="AK5" s="177"/>
+      <c r="AL5" s="177"/>
+      <c r="AM5" s="177"/>
+      <c r="AN5" s="177"/>
+      <c r="AO5" s="177"/>
+      <c r="AP5" s="179" t="s">
         <v>10</v>
       </c>
-      <c r="AQ5" s="89"/>
-      <c r="AR5" s="89"/>
-      <c r="AS5" s="89"/>
-      <c r="AT5" s="89"/>
-      <c r="AU5" s="89"/>
-      <c r="AV5" s="92"/>
+      <c r="AQ5" s="177"/>
+      <c r="AR5" s="177"/>
+      <c r="AS5" s="177"/>
+      <c r="AT5" s="177"/>
+      <c r="AU5" s="177"/>
+      <c r="AV5" s="180"/>
     </row>
     <row r="6" spans="1:50" s="13" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A6" s="81" t="s">
+      <c r="A6" s="169" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="82"/>
-      <c r="C6" s="82"/>
-      <c r="D6" s="82"/>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="83"/>
-      <c r="I6" s="84" t="s">
+      <c r="B6" s="170"/>
+      <c r="C6" s="170"/>
+      <c r="D6" s="170"/>
+      <c r="E6" s="170"/>
+      <c r="F6" s="170"/>
+      <c r="G6" s="170"/>
+      <c r="H6" s="171"/>
+      <c r="I6" s="172" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="82"/>
-      <c r="K6" s="82"/>
-      <c r="L6" s="82"/>
-      <c r="M6" s="82"/>
-      <c r="N6" s="82"/>
-      <c r="O6" s="82"/>
-      <c r="P6" s="82"/>
-      <c r="Q6" s="82"/>
-      <c r="R6" s="82"/>
-      <c r="S6" s="82"/>
-      <c r="T6" s="82"/>
-      <c r="U6" s="84" t="s">
+      <c r="J6" s="170"/>
+      <c r="K6" s="170"/>
+      <c r="L6" s="170"/>
+      <c r="M6" s="170"/>
+      <c r="N6" s="170"/>
+      <c r="O6" s="170"/>
+      <c r="P6" s="170"/>
+      <c r="Q6" s="170"/>
+      <c r="R6" s="170"/>
+      <c r="S6" s="170"/>
+      <c r="T6" s="170"/>
+      <c r="U6" s="172" t="s">
         <v>13</v>
       </c>
-      <c r="V6" s="82"/>
-      <c r="W6" s="82"/>
-      <c r="X6" s="82"/>
-      <c r="Y6" s="82"/>
-      <c r="Z6" s="82"/>
-      <c r="AA6" s="83"/>
-      <c r="AB6" s="84" t="s">
+      <c r="V6" s="170"/>
+      <c r="W6" s="170"/>
+      <c r="X6" s="170"/>
+      <c r="Y6" s="170"/>
+      <c r="Z6" s="170"/>
+      <c r="AA6" s="171"/>
+      <c r="AB6" s="172" t="s">
         <v>14</v>
       </c>
-      <c r="AC6" s="82"/>
-      <c r="AD6" s="82"/>
-      <c r="AE6" s="82"/>
-      <c r="AF6" s="82"/>
-      <c r="AG6" s="82"/>
-      <c r="AH6" s="83"/>
-      <c r="AI6" s="84" t="s">
+      <c r="AC6" s="170"/>
+      <c r="AD6" s="170"/>
+      <c r="AE6" s="170"/>
+      <c r="AF6" s="170"/>
+      <c r="AG6" s="170"/>
+      <c r="AH6" s="171"/>
+      <c r="AI6" s="172" t="s">
         <v>15</v>
       </c>
-      <c r="AJ6" s="82"/>
-      <c r="AK6" s="82"/>
-      <c r="AL6" s="82"/>
-      <c r="AM6" s="82"/>
-      <c r="AN6" s="82"/>
-      <c r="AO6" s="82"/>
-      <c r="AP6" s="84" t="s">
+      <c r="AJ6" s="170"/>
+      <c r="AK6" s="170"/>
+      <c r="AL6" s="170"/>
+      <c r="AM6" s="170"/>
+      <c r="AN6" s="170"/>
+      <c r="AO6" s="170"/>
+      <c r="AP6" s="172" t="s">
         <v>16</v>
       </c>
-      <c r="AQ6" s="82"/>
-      <c r="AR6" s="82"/>
-      <c r="AS6" s="82"/>
-      <c r="AT6" s="82"/>
-      <c r="AU6" s="82"/>
-      <c r="AV6" s="85"/>
+      <c r="AQ6" s="170"/>
+      <c r="AR6" s="170"/>
+      <c r="AS6" s="170"/>
+      <c r="AT6" s="170"/>
+      <c r="AU6" s="170"/>
+      <c r="AV6" s="173"/>
     </row>
     <row r="7" spans="1:50" s="13" customFormat="1" ht="34.15" customHeight="1" thickBot="1">
-      <c r="A7" s="114"/>
-      <c r="B7" s="115"/>
-      <c r="C7" s="115"/>
-      <c r="D7" s="115"/>
-      <c r="E7" s="115"/>
-      <c r="F7" s="115"/>
-      <c r="G7" s="115"/>
-      <c r="H7" s="115"/>
-      <c r="I7" s="116"/>
-      <c r="J7" s="115"/>
-      <c r="K7" s="115"/>
-      <c r="L7" s="115"/>
-      <c r="M7" s="115"/>
-      <c r="N7" s="115"/>
-      <c r="O7" s="115"/>
-      <c r="P7" s="115"/>
-      <c r="Q7" s="115"/>
-      <c r="R7" s="115"/>
-      <c r="S7" s="115"/>
-      <c r="T7" s="117"/>
-      <c r="U7" s="118"/>
-      <c r="V7" s="119"/>
-      <c r="W7" s="119"/>
-      <c r="X7" s="119"/>
-      <c r="Y7" s="119"/>
-      <c r="Z7" s="119"/>
-      <c r="AA7" s="120"/>
-      <c r="AB7" s="118"/>
-      <c r="AC7" s="119"/>
-      <c r="AD7" s="119"/>
-      <c r="AE7" s="119"/>
-      <c r="AF7" s="119"/>
-      <c r="AG7" s="119"/>
-      <c r="AH7" s="120"/>
-      <c r="AI7" s="118"/>
-      <c r="AJ7" s="119"/>
-      <c r="AK7" s="119"/>
-      <c r="AL7" s="119"/>
-      <c r="AM7" s="119"/>
-      <c r="AN7" s="119"/>
-      <c r="AO7" s="119"/>
-      <c r="AP7" s="121"/>
-      <c r="AQ7" s="122"/>
-      <c r="AR7" s="122"/>
-      <c r="AS7" s="122"/>
-      <c r="AT7" s="122"/>
-      <c r="AU7" s="122"/>
-      <c r="AV7" s="123"/>
+      <c r="A7" s="159"/>
+      <c r="B7" s="160"/>
+      <c r="C7" s="160"/>
+      <c r="D7" s="160"/>
+      <c r="E7" s="160"/>
+      <c r="F7" s="160"/>
+      <c r="G7" s="160"/>
+      <c r="H7" s="160"/>
+      <c r="I7" s="161"/>
+      <c r="J7" s="160"/>
+      <c r="K7" s="160"/>
+      <c r="L7" s="160"/>
+      <c r="M7" s="160"/>
+      <c r="N7" s="160"/>
+      <c r="O7" s="160"/>
+      <c r="P7" s="160"/>
+      <c r="Q7" s="160"/>
+      <c r="R7" s="160"/>
+      <c r="S7" s="160"/>
+      <c r="T7" s="162"/>
+      <c r="U7" s="163"/>
+      <c r="V7" s="164"/>
+      <c r="W7" s="164"/>
+      <c r="X7" s="164"/>
+      <c r="Y7" s="164"/>
+      <c r="Z7" s="164"/>
+      <c r="AA7" s="165"/>
+      <c r="AB7" s="163"/>
+      <c r="AC7" s="164"/>
+      <c r="AD7" s="164"/>
+      <c r="AE7" s="164"/>
+      <c r="AF7" s="164"/>
+      <c r="AG7" s="164"/>
+      <c r="AH7" s="165"/>
+      <c r="AI7" s="163"/>
+      <c r="AJ7" s="164"/>
+      <c r="AK7" s="164"/>
+      <c r="AL7" s="164"/>
+      <c r="AM7" s="164"/>
+      <c r="AN7" s="164"/>
+      <c r="AO7" s="164"/>
+      <c r="AP7" s="166"/>
+      <c r="AQ7" s="167"/>
+      <c r="AR7" s="167"/>
+      <c r="AS7" s="167"/>
+      <c r="AT7" s="167"/>
+      <c r="AU7" s="167"/>
+      <c r="AV7" s="168"/>
     </row>
     <row r="8" spans="1:50" s="13" customFormat="1" ht="36.75" customHeight="1" thickTop="1">
       <c r="A8" s="64" t="s">
@@ -2744,34 +2753,34 @@
       <c r="Z8" s="65"/>
       <c r="AA8" s="20"/>
       <c r="AB8" s="20"/>
-      <c r="AC8" s="93" t="s">
+      <c r="AC8" s="91" t="s">
         <v>19</v>
       </c>
-      <c r="AD8" s="94"/>
-      <c r="AE8" s="95"/>
+      <c r="AD8" s="90"/>
+      <c r="AE8" s="147"/>
       <c r="AF8" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="AG8" s="96" t="s">
+      <c r="AG8" s="148" t="s">
         <v>21</v>
       </c>
-      <c r="AH8" s="96"/>
-      <c r="AI8" s="96"/>
-      <c r="AJ8" s="96"/>
-      <c r="AK8" s="96"/>
-      <c r="AL8" s="96"/>
-      <c r="AM8" s="96"/>
-      <c r="AN8" s="96"/>
-      <c r="AO8" s="96"/>
-      <c r="AP8" s="96"/>
-      <c r="AQ8" s="96"/>
-      <c r="AR8" s="96"/>
-      <c r="AS8" s="97"/>
-      <c r="AT8" s="93" t="s">
+      <c r="AH8" s="148"/>
+      <c r="AI8" s="148"/>
+      <c r="AJ8" s="148"/>
+      <c r="AK8" s="148"/>
+      <c r="AL8" s="148"/>
+      <c r="AM8" s="148"/>
+      <c r="AN8" s="148"/>
+      <c r="AO8" s="148"/>
+      <c r="AP8" s="148"/>
+      <c r="AQ8" s="148"/>
+      <c r="AR8" s="148"/>
+      <c r="AS8" s="149"/>
+      <c r="AT8" s="91" t="s">
         <v>19</v>
       </c>
-      <c r="AU8" s="94"/>
-      <c r="AV8" s="98"/>
+      <c r="AU8" s="90"/>
+      <c r="AV8" s="92"/>
     </row>
     <row r="9" spans="1:50" s="13" customFormat="1" ht="21.6" customHeight="1">
       <c r="A9" s="37" t="s">
@@ -2808,9 +2817,9 @@
       <c r="Z9" s="67"/>
       <c r="AA9" s="67"/>
       <c r="AB9" s="67"/>
-      <c r="AC9" s="99"/>
-      <c r="AD9" s="99"/>
-      <c r="AE9" s="100"/>
+      <c r="AC9" s="150"/>
+      <c r="AD9" s="150"/>
+      <c r="AE9" s="151"/>
       <c r="AF9" s="31" t="s">
         <v>25</v>
       </c>
@@ -2862,9 +2871,9 @@
       <c r="Z10" s="69"/>
       <c r="AA10" s="69"/>
       <c r="AB10" s="69"/>
-      <c r="AC10" s="99"/>
-      <c r="AD10" s="99"/>
-      <c r="AE10" s="100"/>
+      <c r="AC10" s="150"/>
+      <c r="AD10" s="150"/>
+      <c r="AE10" s="151"/>
       <c r="AF10" s="33"/>
       <c r="AG10" s="21" t="s">
         <v>27</v>
@@ -2914,9 +2923,9 @@
       <c r="Z11" s="27"/>
       <c r="AA11" s="27"/>
       <c r="AB11" s="27"/>
-      <c r="AC11" s="99"/>
-      <c r="AD11" s="99"/>
-      <c r="AE11" s="100"/>
+      <c r="AC11" s="150"/>
+      <c r="AD11" s="150"/>
+      <c r="AE11" s="151"/>
       <c r="AF11" s="72" t="s">
         <v>28</v>
       </c>
@@ -2968,9 +2977,9 @@
       <c r="Z12" s="31"/>
       <c r="AA12" s="31"/>
       <c r="AB12" s="31"/>
-      <c r="AC12" s="99"/>
-      <c r="AD12" s="99"/>
-      <c r="AE12" s="100"/>
+      <c r="AC12" s="150"/>
+      <c r="AD12" s="150"/>
+      <c r="AE12" s="151"/>
       <c r="AF12" s="30"/>
       <c r="AG12" s="21" t="s">
         <v>30</v>
@@ -3026,9 +3035,9 @@
       <c r="Z13" s="80"/>
       <c r="AA13" s="80"/>
       <c r="AB13" s="80"/>
-      <c r="AC13" s="101"/>
-      <c r="AD13" s="102"/>
-      <c r="AE13" s="103"/>
+      <c r="AC13" s="123"/>
+      <c r="AD13" s="124"/>
+      <c r="AE13" s="125"/>
       <c r="AF13" s="73" t="s">
         <v>34</v>
       </c>
@@ -3080,9 +3089,9 @@
       <c r="Z14" s="27"/>
       <c r="AA14" s="27"/>
       <c r="AB14" s="27"/>
-      <c r="AC14" s="104"/>
-      <c r="AD14" s="105"/>
-      <c r="AE14" s="106"/>
+      <c r="AC14" s="126"/>
+      <c r="AD14" s="127"/>
+      <c r="AE14" s="128"/>
       <c r="AF14" s="33"/>
       <c r="AG14" s="21" t="s">
         <v>36</v>
@@ -3132,9 +3141,9 @@
       <c r="Z15" s="30"/>
       <c r="AA15" s="30"/>
       <c r="AB15" s="30"/>
-      <c r="AC15" s="104"/>
-      <c r="AD15" s="105"/>
-      <c r="AE15" s="106"/>
+      <c r="AC15" s="126"/>
+      <c r="AD15" s="127"/>
+      <c r="AE15" s="128"/>
       <c r="AF15" s="74" t="s">
         <v>37</v>
       </c>
@@ -3186,25 +3195,25 @@
       <c r="Z16" s="30"/>
       <c r="AA16" s="30"/>
       <c r="AB16" s="30"/>
-      <c r="AC16" s="104"/>
-      <c r="AD16" s="105"/>
-      <c r="AE16" s="106"/>
+      <c r="AC16" s="126"/>
+      <c r="AD16" s="127"/>
+      <c r="AE16" s="128"/>
       <c r="AF16" s="35"/>
-      <c r="AG16" s="110" t="s">
+      <c r="AG16" s="155" t="s">
         <v>39</v>
       </c>
-      <c r="AH16" s="110"/>
-      <c r="AI16" s="110"/>
-      <c r="AJ16" s="110"/>
-      <c r="AK16" s="110"/>
-      <c r="AL16" s="110"/>
-      <c r="AM16" s="110"/>
-      <c r="AN16" s="110"/>
-      <c r="AO16" s="110"/>
-      <c r="AP16" s="110"/>
-      <c r="AQ16" s="110"/>
-      <c r="AR16" s="110"/>
-      <c r="AS16" s="111"/>
+      <c r="AH16" s="155"/>
+      <c r="AI16" s="155"/>
+      <c r="AJ16" s="155"/>
+      <c r="AK16" s="155"/>
+      <c r="AL16" s="155"/>
+      <c r="AM16" s="155"/>
+      <c r="AN16" s="155"/>
+      <c r="AO16" s="155"/>
+      <c r="AP16" s="155"/>
+      <c r="AQ16" s="155"/>
+      <c r="AR16" s="155"/>
+      <c r="AS16" s="156"/>
       <c r="AT16" s="24"/>
       <c r="AU16" s="22"/>
       <c r="AV16" s="25"/>
@@ -3239,9 +3248,9 @@
       <c r="Z17" s="27"/>
       <c r="AA17" s="27"/>
       <c r="AB17" s="27"/>
-      <c r="AC17" s="107"/>
-      <c r="AD17" s="108"/>
-      <c r="AE17" s="109"/>
+      <c r="AC17" s="152"/>
+      <c r="AD17" s="153"/>
+      <c r="AE17" s="154"/>
       <c r="AF17" s="72" t="s">
         <v>40</v>
       </c>
@@ -3260,9 +3269,9 @@
       <c r="AQ17" s="28"/>
       <c r="AR17" s="28"/>
       <c r="AS17" s="28"/>
-      <c r="AT17" s="101"/>
-      <c r="AU17" s="102"/>
-      <c r="AV17" s="112"/>
+      <c r="AT17" s="123"/>
+      <c r="AU17" s="124"/>
+      <c r="AV17" s="157"/>
       <c r="AX17" s="27"/>
     </row>
     <row r="18" spans="1:50" s="13" customFormat="1" ht="21" customHeight="1">
@@ -3300,9 +3309,9 @@
       <c r="Z18" s="71"/>
       <c r="AA18" s="71"/>
       <c r="AB18" s="71"/>
-      <c r="AC18" s="101"/>
-      <c r="AD18" s="102"/>
-      <c r="AE18" s="103"/>
+      <c r="AC18" s="123"/>
+      <c r="AD18" s="124"/>
+      <c r="AE18" s="125"/>
       <c r="AF18" s="35"/>
       <c r="AG18" s="21" t="s">
         <v>45</v>
@@ -3319,9 +3328,9 @@
       <c r="AQ18" s="21"/>
       <c r="AR18" s="21"/>
       <c r="AS18" s="21"/>
-      <c r="AT18" s="107"/>
-      <c r="AU18" s="108"/>
-      <c r="AV18" s="113"/>
+      <c r="AT18" s="152"/>
+      <c r="AU18" s="153"/>
+      <c r="AV18" s="158"/>
     </row>
     <row r="19" spans="1:50" s="13" customFormat="1" ht="20.25" customHeight="1">
       <c r="A19" s="37"/>
@@ -3352,9 +3361,9 @@
       <c r="Z19" s="30"/>
       <c r="AA19" s="30"/>
       <c r="AB19" s="30"/>
-      <c r="AC19" s="104"/>
-      <c r="AD19" s="105"/>
-      <c r="AE19" s="106"/>
+      <c r="AC19" s="126"/>
+      <c r="AD19" s="127"/>
+      <c r="AE19" s="128"/>
       <c r="AF19" s="72" t="s">
         <v>46</v>
       </c>
@@ -3406,9 +3415,9 @@
       <c r="Z20" s="30"/>
       <c r="AA20" s="30"/>
       <c r="AB20" s="30"/>
-      <c r="AC20" s="104"/>
-      <c r="AD20" s="105"/>
-      <c r="AE20" s="106"/>
+      <c r="AC20" s="126"/>
+      <c r="AD20" s="127"/>
+      <c r="AE20" s="128"/>
       <c r="AF20" s="35"/>
       <c r="AG20" s="21" t="s">
         <v>48</v>
@@ -3458,9 +3467,9 @@
       <c r="Z21" s="30"/>
       <c r="AA21" s="30"/>
       <c r="AB21" s="30"/>
-      <c r="AC21" s="104"/>
-      <c r="AD21" s="105"/>
-      <c r="AE21" s="106"/>
+      <c r="AC21" s="126"/>
+      <c r="AD21" s="127"/>
+      <c r="AE21" s="128"/>
       <c r="AF21" s="72" t="s">
         <v>49</v>
       </c>
@@ -3512,9 +3521,9 @@
       <c r="Z22" s="30"/>
       <c r="AA22" s="30"/>
       <c r="AB22" s="30"/>
-      <c r="AC22" s="107"/>
-      <c r="AD22" s="108"/>
-      <c r="AE22" s="109"/>
+      <c r="AC22" s="152"/>
+      <c r="AD22" s="153"/>
+      <c r="AE22" s="154"/>
       <c r="AF22" s="76"/>
       <c r="AG22" s="21" t="s">
         <v>51</v>
@@ -3570,27 +3579,27 @@
       <c r="Z23" s="71"/>
       <c r="AA23" s="71"/>
       <c r="AB23" s="71"/>
-      <c r="AC23" s="101"/>
-      <c r="AD23" s="102"/>
-      <c r="AE23" s="103"/>
+      <c r="AC23" s="123"/>
+      <c r="AD23" s="124"/>
+      <c r="AE23" s="125"/>
       <c r="AF23" s="73" t="s">
         <v>55</v>
       </c>
-      <c r="AG23" s="127" t="s">
+      <c r="AG23" s="132" t="s">
         <v>56</v>
       </c>
-      <c r="AH23" s="127"/>
-      <c r="AI23" s="127"/>
-      <c r="AJ23" s="127"/>
-      <c r="AK23" s="127"/>
-      <c r="AL23" s="127"/>
-      <c r="AM23" s="127"/>
-      <c r="AN23" s="127"/>
-      <c r="AO23" s="127"/>
-      <c r="AP23" s="127"/>
-      <c r="AQ23" s="127"/>
-      <c r="AR23" s="127"/>
-      <c r="AS23" s="128"/>
+      <c r="AH23" s="132"/>
+      <c r="AI23" s="132"/>
+      <c r="AJ23" s="132"/>
+      <c r="AK23" s="132"/>
+      <c r="AL23" s="132"/>
+      <c r="AM23" s="132"/>
+      <c r="AN23" s="132"/>
+      <c r="AO23" s="132"/>
+      <c r="AP23" s="132"/>
+      <c r="AQ23" s="132"/>
+      <c r="AR23" s="132"/>
+      <c r="AS23" s="133"/>
       <c r="AT23" s="18"/>
       <c r="AU23" s="16"/>
       <c r="AV23" s="19"/>
@@ -3624,25 +3633,25 @@
       <c r="Z24" s="27"/>
       <c r="AA24" s="27"/>
       <c r="AB24" s="27"/>
-      <c r="AC24" s="104"/>
-      <c r="AD24" s="105"/>
-      <c r="AE24" s="106"/>
+      <c r="AC24" s="126"/>
+      <c r="AD24" s="127"/>
+      <c r="AE24" s="128"/>
       <c r="AF24" s="33"/>
-      <c r="AG24" s="129" t="s">
+      <c r="AG24" s="134" t="s">
         <v>57</v>
       </c>
-      <c r="AH24" s="129"/>
-      <c r="AI24" s="129"/>
-      <c r="AJ24" s="129"/>
-      <c r="AK24" s="129"/>
-      <c r="AL24" s="129"/>
-      <c r="AM24" s="129"/>
-      <c r="AN24" s="129"/>
-      <c r="AO24" s="129"/>
-      <c r="AP24" s="129"/>
-      <c r="AQ24" s="129"/>
-      <c r="AR24" s="129"/>
-      <c r="AS24" s="130"/>
+      <c r="AH24" s="134"/>
+      <c r="AI24" s="134"/>
+      <c r="AJ24" s="134"/>
+      <c r="AK24" s="134"/>
+      <c r="AL24" s="134"/>
+      <c r="AM24" s="134"/>
+      <c r="AN24" s="134"/>
+      <c r="AO24" s="134"/>
+      <c r="AP24" s="134"/>
+      <c r="AQ24" s="134"/>
+      <c r="AR24" s="134"/>
+      <c r="AS24" s="135"/>
       <c r="AT24" s="24"/>
       <c r="AU24" s="22"/>
       <c r="AV24" s="25"/>
@@ -3676,27 +3685,27 @@
       <c r="Z25" s="27"/>
       <c r="AA25" s="27"/>
       <c r="AB25" s="27"/>
-      <c r="AC25" s="104"/>
-      <c r="AD25" s="105"/>
-      <c r="AE25" s="106"/>
+      <c r="AC25" s="126"/>
+      <c r="AD25" s="127"/>
+      <c r="AE25" s="128"/>
       <c r="AF25" s="73" t="s">
         <v>58</v>
       </c>
-      <c r="AG25" s="127" t="s">
+      <c r="AG25" s="132" t="s">
         <v>59</v>
       </c>
-      <c r="AH25" s="127"/>
-      <c r="AI25" s="127"/>
-      <c r="AJ25" s="127"/>
-      <c r="AK25" s="127"/>
-      <c r="AL25" s="127"/>
-      <c r="AM25" s="127"/>
-      <c r="AN25" s="127"/>
-      <c r="AO25" s="127"/>
-      <c r="AP25" s="127"/>
-      <c r="AQ25" s="127"/>
-      <c r="AR25" s="127"/>
-      <c r="AS25" s="128"/>
+      <c r="AH25" s="132"/>
+      <c r="AI25" s="132"/>
+      <c r="AJ25" s="132"/>
+      <c r="AK25" s="132"/>
+      <c r="AL25" s="132"/>
+      <c r="AM25" s="132"/>
+      <c r="AN25" s="132"/>
+      <c r="AO25" s="132"/>
+      <c r="AP25" s="132"/>
+      <c r="AQ25" s="132"/>
+      <c r="AR25" s="132"/>
+      <c r="AS25" s="133"/>
       <c r="AT25" s="18"/>
       <c r="AU25" s="27"/>
       <c r="AV25" s="40"/>
@@ -3730,25 +3739,25 @@
       <c r="Z26" s="42"/>
       <c r="AA26" s="42"/>
       <c r="AB26" s="42"/>
-      <c r="AC26" s="124"/>
-      <c r="AD26" s="125"/>
-      <c r="AE26" s="126"/>
+      <c r="AC26" s="129"/>
+      <c r="AD26" s="130"/>
+      <c r="AE26" s="131"/>
       <c r="AF26" s="43"/>
-      <c r="AG26" s="131" t="s">
+      <c r="AG26" s="136" t="s">
         <v>60</v>
       </c>
-      <c r="AH26" s="131"/>
-      <c r="AI26" s="131"/>
-      <c r="AJ26" s="131"/>
-      <c r="AK26" s="131"/>
-      <c r="AL26" s="131"/>
-      <c r="AM26" s="131"/>
-      <c r="AN26" s="131"/>
-      <c r="AO26" s="131"/>
-      <c r="AP26" s="131"/>
-      <c r="AQ26" s="131"/>
-      <c r="AR26" s="131"/>
-      <c r="AS26" s="132"/>
+      <c r="AH26" s="136"/>
+      <c r="AI26" s="136"/>
+      <c r="AJ26" s="136"/>
+      <c r="AK26" s="136"/>
+      <c r="AL26" s="136"/>
+      <c r="AM26" s="136"/>
+      <c r="AN26" s="136"/>
+      <c r="AO26" s="136"/>
+      <c r="AP26" s="136"/>
+      <c r="AQ26" s="136"/>
+      <c r="AR26" s="136"/>
+      <c r="AS26" s="137"/>
       <c r="AT26" s="44"/>
       <c r="AU26" s="42"/>
       <c r="AV26" s="45"/>
@@ -3806,154 +3815,154 @@
       <c r="AV27" s="40"/>
     </row>
     <row r="28" spans="1:50" s="13" customFormat="1" ht="21.75" customHeight="1">
-      <c r="A28" s="133" t="s">
+      <c r="A28" s="138" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="134"/>
-      <c r="C28" s="137" t="s">
+      <c r="B28" s="139"/>
+      <c r="C28" s="112" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="138"/>
-      <c r="E28" s="138"/>
-      <c r="F28" s="138"/>
-      <c r="G28" s="139"/>
-      <c r="H28" s="143" t="s">
+      <c r="D28" s="113"/>
+      <c r="E28" s="113"/>
+      <c r="F28" s="113"/>
+      <c r="G28" s="114"/>
+      <c r="H28" s="142" t="s">
         <v>64</v>
       </c>
-      <c r="I28" s="143"/>
-      <c r="J28" s="143"/>
-      <c r="K28" s="144" t="s">
+      <c r="I28" s="142"/>
+      <c r="J28" s="142"/>
+      <c r="K28" s="143" t="s">
         <v>65</v>
       </c>
-      <c r="L28" s="145"/>
-      <c r="M28" s="145"/>
-      <c r="N28" s="145"/>
-      <c r="O28" s="145"/>
-      <c r="P28" s="145"/>
-      <c r="Q28" s="145"/>
-      <c r="R28" s="145"/>
-      <c r="S28" s="145"/>
-      <c r="T28" s="145"/>
-      <c r="U28" s="145"/>
-      <c r="V28" s="145"/>
-      <c r="W28" s="145"/>
-      <c r="X28" s="146"/>
-      <c r="Y28" s="147" t="s">
+      <c r="L28" s="119"/>
+      <c r="M28" s="119"/>
+      <c r="N28" s="119"/>
+      <c r="O28" s="119"/>
+      <c r="P28" s="119"/>
+      <c r="Q28" s="119"/>
+      <c r="R28" s="119"/>
+      <c r="S28" s="119"/>
+      <c r="T28" s="119"/>
+      <c r="U28" s="119"/>
+      <c r="V28" s="119"/>
+      <c r="W28" s="119"/>
+      <c r="X28" s="144"/>
+      <c r="Y28" s="145" t="s">
         <v>62</v>
       </c>
-      <c r="Z28" s="134"/>
-      <c r="AA28" s="137" t="s">
+      <c r="Z28" s="139"/>
+      <c r="AA28" s="112" t="s">
         <v>66</v>
       </c>
-      <c r="AB28" s="138"/>
-      <c r="AC28" s="138"/>
-      <c r="AD28" s="138"/>
-      <c r="AE28" s="139"/>
-      <c r="AF28" s="164" t="s">
+      <c r="AB28" s="113"/>
+      <c r="AC28" s="113"/>
+      <c r="AD28" s="113"/>
+      <c r="AE28" s="114"/>
+      <c r="AF28" s="118" t="s">
         <v>64</v>
       </c>
-      <c r="AG28" s="164"/>
-      <c r="AH28" s="164"/>
-      <c r="AI28" s="145" t="s">
+      <c r="AG28" s="118"/>
+      <c r="AH28" s="118"/>
+      <c r="AI28" s="119" t="s">
         <v>67</v>
       </c>
-      <c r="AJ28" s="145"/>
-      <c r="AK28" s="145"/>
-      <c r="AL28" s="145"/>
-      <c r="AM28" s="145"/>
-      <c r="AN28" s="145"/>
-      <c r="AO28" s="145"/>
-      <c r="AP28" s="145"/>
-      <c r="AQ28" s="145"/>
-      <c r="AR28" s="145"/>
-      <c r="AS28" s="145"/>
-      <c r="AT28" s="145"/>
-      <c r="AU28" s="145"/>
-      <c r="AV28" s="165"/>
+      <c r="AJ28" s="119"/>
+      <c r="AK28" s="119"/>
+      <c r="AL28" s="119"/>
+      <c r="AM28" s="119"/>
+      <c r="AN28" s="119"/>
+      <c r="AO28" s="119"/>
+      <c r="AP28" s="119"/>
+      <c r="AQ28" s="119"/>
+      <c r="AR28" s="119"/>
+      <c r="AS28" s="119"/>
+      <c r="AT28" s="119"/>
+      <c r="AU28" s="119"/>
+      <c r="AV28" s="120"/>
     </row>
     <row r="29" spans="1:50" s="13" customFormat="1" ht="39.75" customHeight="1">
-      <c r="A29" s="135"/>
-      <c r="B29" s="136"/>
-      <c r="C29" s="140"/>
-      <c r="D29" s="141"/>
-      <c r="E29" s="141"/>
-      <c r="F29" s="141"/>
-      <c r="G29" s="142"/>
-      <c r="H29" s="143"/>
-      <c r="I29" s="143"/>
-      <c r="J29" s="143"/>
-      <c r="K29" s="149" t="s">
+      <c r="A29" s="140"/>
+      <c r="B29" s="141"/>
+      <c r="C29" s="115"/>
+      <c r="D29" s="116"/>
+      <c r="E29" s="116"/>
+      <c r="F29" s="116"/>
+      <c r="G29" s="117"/>
+      <c r="H29" s="142"/>
+      <c r="I29" s="142"/>
+      <c r="J29" s="142"/>
+      <c r="K29" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="L29" s="151"/>
-      <c r="M29" s="149" t="s">
+      <c r="L29" s="121"/>
+      <c r="M29" s="108" t="s">
         <v>31</v>
       </c>
-      <c r="N29" s="150"/>
-      <c r="O29" s="151"/>
-      <c r="P29" s="149" t="s">
+      <c r="N29" s="109"/>
+      <c r="O29" s="121"/>
+      <c r="P29" s="108" t="s">
         <v>42</v>
       </c>
-      <c r="Q29" s="150"/>
-      <c r="R29" s="151"/>
-      <c r="S29" s="149" t="s">
+      <c r="Q29" s="109"/>
+      <c r="R29" s="121"/>
+      <c r="S29" s="108" t="s">
         <v>52</v>
       </c>
-      <c r="T29" s="150"/>
-      <c r="U29" s="151"/>
-      <c r="V29" s="149" t="s">
+      <c r="T29" s="109"/>
+      <c r="U29" s="121"/>
+      <c r="V29" s="108" t="s">
         <v>68</v>
       </c>
-      <c r="W29" s="150"/>
-      <c r="X29" s="166"/>
-      <c r="Y29" s="148"/>
-      <c r="Z29" s="136"/>
-      <c r="AA29" s="140"/>
-      <c r="AB29" s="141"/>
-      <c r="AC29" s="141"/>
-      <c r="AD29" s="141"/>
-      <c r="AE29" s="142"/>
-      <c r="AF29" s="164"/>
-      <c r="AG29" s="164"/>
-      <c r="AH29" s="164"/>
-      <c r="AI29" s="150" t="s">
+      <c r="W29" s="109"/>
+      <c r="X29" s="122"/>
+      <c r="Y29" s="146"/>
+      <c r="Z29" s="141"/>
+      <c r="AA29" s="115"/>
+      <c r="AB29" s="116"/>
+      <c r="AC29" s="116"/>
+      <c r="AD29" s="116"/>
+      <c r="AE29" s="117"/>
+      <c r="AF29" s="118"/>
+      <c r="AG29" s="118"/>
+      <c r="AH29" s="118"/>
+      <c r="AI29" s="109" t="s">
         <v>25</v>
       </c>
-      <c r="AJ29" s="151"/>
-      <c r="AK29" s="149" t="s">
+      <c r="AJ29" s="121"/>
+      <c r="AK29" s="108" t="s">
         <v>31</v>
       </c>
-      <c r="AL29" s="150"/>
-      <c r="AM29" s="151"/>
-      <c r="AN29" s="149" t="s">
+      <c r="AL29" s="109"/>
+      <c r="AM29" s="121"/>
+      <c r="AN29" s="108" t="s">
         <v>42</v>
       </c>
-      <c r="AO29" s="150"/>
-      <c r="AP29" s="151"/>
-      <c r="AQ29" s="149" t="s">
+      <c r="AO29" s="109"/>
+      <c r="AP29" s="121"/>
+      <c r="AQ29" s="108" t="s">
         <v>52</v>
       </c>
-      <c r="AR29" s="150"/>
-      <c r="AS29" s="151"/>
-      <c r="AT29" s="149" t="s">
+      <c r="AR29" s="109"/>
+      <c r="AS29" s="121"/>
+      <c r="AT29" s="108" t="s">
         <v>68</v>
       </c>
-      <c r="AU29" s="150"/>
-      <c r="AV29" s="152"/>
+      <c r="AU29" s="109"/>
+      <c r="AV29" s="110"/>
     </row>
     <row r="30" spans="1:50" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A30" s="153">
+      <c r="A30" s="95">
         <v>1</v>
       </c>
-      <c r="B30" s="154"/>
-      <c r="C30" s="155"/>
-      <c r="D30" s="156"/>
-      <c r="E30" s="156"/>
-      <c r="F30" s="156"/>
-      <c r="G30" s="157"/>
-      <c r="H30" s="158"/>
-      <c r="I30" s="158"/>
-      <c r="J30" s="158"/>
+      <c r="B30" s="96"/>
+      <c r="C30" s="97"/>
+      <c r="D30" s="98"/>
+      <c r="E30" s="98"/>
+      <c r="F30" s="98"/>
+      <c r="G30" s="99"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
       <c r="K30" s="47"/>
       <c r="L30" s="48"/>
       <c r="M30" s="49"/>
@@ -3968,20 +3977,20 @@
       <c r="V30" s="49"/>
       <c r="W30" s="47"/>
       <c r="X30" s="50"/>
-      <c r="Y30" s="159">
+      <c r="Y30" s="101">
         <v>12</v>
       </c>
-      <c r="Z30" s="154"/>
-      <c r="AA30" s="160"/>
-      <c r="AB30" s="160"/>
-      <c r="AC30" s="160"/>
-      <c r="AD30" s="160"/>
-      <c r="AE30" s="160"/>
-      <c r="AF30" s="161"/>
-      <c r="AG30" s="161"/>
-      <c r="AH30" s="161"/>
-      <c r="AI30" s="162"/>
-      <c r="AJ30" s="163"/>
+      <c r="Z30" s="96"/>
+      <c r="AA30" s="111"/>
+      <c r="AB30" s="111"/>
+      <c r="AC30" s="111"/>
+      <c r="AD30" s="111"/>
+      <c r="AE30" s="111"/>
+      <c r="AF30" s="106"/>
+      <c r="AG30" s="106"/>
+      <c r="AH30" s="106"/>
+      <c r="AI30" s="93"/>
+      <c r="AJ30" s="94"/>
       <c r="AK30" s="49"/>
       <c r="AL30" s="47"/>
       <c r="AM30" s="48"/>
@@ -3996,18 +4005,18 @@
       <c r="AV30" s="51"/>
     </row>
     <row r="31" spans="1:50" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A31" s="153">
+      <c r="A31" s="95">
         <v>2</v>
       </c>
-      <c r="B31" s="154"/>
-      <c r="C31" s="155"/>
-      <c r="D31" s="156"/>
-      <c r="E31" s="156"/>
-      <c r="F31" s="156"/>
-      <c r="G31" s="157"/>
-      <c r="H31" s="158"/>
-      <c r="I31" s="158"/>
-      <c r="J31" s="158"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="97"/>
+      <c r="D31" s="98"/>
+      <c r="E31" s="98"/>
+      <c r="F31" s="98"/>
+      <c r="G31" s="99"/>
+      <c r="H31" s="100"/>
+      <c r="I31" s="100"/>
+      <c r="J31" s="100"/>
       <c r="K31" s="47"/>
       <c r="L31" s="48"/>
       <c r="M31" s="49"/>
@@ -4022,20 +4031,20 @@
       <c r="V31" s="49"/>
       <c r="W31" s="47"/>
       <c r="X31" s="50"/>
-      <c r="Y31" s="159">
+      <c r="Y31" s="101">
         <v>13</v>
       </c>
-      <c r="Z31" s="154"/>
-      <c r="AA31" s="167"/>
-      <c r="AB31" s="167"/>
-      <c r="AC31" s="167"/>
-      <c r="AD31" s="167"/>
-      <c r="AE31" s="167"/>
-      <c r="AF31" s="168"/>
-      <c r="AG31" s="168"/>
-      <c r="AH31" s="168"/>
-      <c r="AI31" s="162"/>
-      <c r="AJ31" s="163"/>
+      <c r="Z31" s="96"/>
+      <c r="AA31" s="105"/>
+      <c r="AB31" s="105"/>
+      <c r="AC31" s="105"/>
+      <c r="AD31" s="105"/>
+      <c r="AE31" s="105"/>
+      <c r="AF31" s="107"/>
+      <c r="AG31" s="107"/>
+      <c r="AH31" s="107"/>
+      <c r="AI31" s="93"/>
+      <c r="AJ31" s="94"/>
       <c r="AK31" s="49"/>
       <c r="AL31" s="47"/>
       <c r="AM31" s="48"/>
@@ -4050,18 +4059,18 @@
       <c r="AV31" s="51"/>
     </row>
     <row r="32" spans="1:50" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A32" s="153">
+      <c r="A32" s="95">
         <v>3</v>
       </c>
-      <c r="B32" s="154"/>
-      <c r="C32" s="155"/>
-      <c r="D32" s="156"/>
-      <c r="E32" s="156"/>
-      <c r="F32" s="156"/>
-      <c r="G32" s="157"/>
-      <c r="H32" s="158"/>
-      <c r="I32" s="158"/>
-      <c r="J32" s="158"/>
+      <c r="B32" s="96"/>
+      <c r="C32" s="97"/>
+      <c r="D32" s="98"/>
+      <c r="E32" s="98"/>
+      <c r="F32" s="98"/>
+      <c r="G32" s="99"/>
+      <c r="H32" s="100"/>
+      <c r="I32" s="100"/>
+      <c r="J32" s="100"/>
       <c r="K32" s="47"/>
       <c r="L32" s="48"/>
       <c r="M32" s="49"/>
@@ -4076,20 +4085,20 @@
       <c r="V32" s="49"/>
       <c r="W32" s="47"/>
       <c r="X32" s="50"/>
-      <c r="Y32" s="159">
+      <c r="Y32" s="101">
         <v>14</v>
       </c>
-      <c r="Z32" s="154"/>
-      <c r="AA32" s="167"/>
-      <c r="AB32" s="167"/>
-      <c r="AC32" s="167"/>
-      <c r="AD32" s="167"/>
-      <c r="AE32" s="167"/>
-      <c r="AF32" s="168"/>
-      <c r="AG32" s="168"/>
-      <c r="AH32" s="168"/>
-      <c r="AI32" s="162"/>
-      <c r="AJ32" s="163"/>
+      <c r="Z32" s="96"/>
+      <c r="AA32" s="105"/>
+      <c r="AB32" s="105"/>
+      <c r="AC32" s="105"/>
+      <c r="AD32" s="105"/>
+      <c r="AE32" s="105"/>
+      <c r="AF32" s="107"/>
+      <c r="AG32" s="107"/>
+      <c r="AH32" s="107"/>
+      <c r="AI32" s="93"/>
+      <c r="AJ32" s="94"/>
       <c r="AK32" s="49"/>
       <c r="AL32" s="47"/>
       <c r="AM32" s="48"/>
@@ -4104,18 +4113,18 @@
       <c r="AV32" s="51"/>
     </row>
     <row r="33" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A33" s="153">
+      <c r="A33" s="95">
         <v>4</v>
       </c>
-      <c r="B33" s="154"/>
-      <c r="C33" s="155"/>
-      <c r="D33" s="156"/>
-      <c r="E33" s="156"/>
-      <c r="F33" s="156"/>
-      <c r="G33" s="157"/>
-      <c r="H33" s="158"/>
-      <c r="I33" s="158"/>
-      <c r="J33" s="158"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="97"/>
+      <c r="D33" s="98"/>
+      <c r="E33" s="98"/>
+      <c r="F33" s="98"/>
+      <c r="G33" s="99"/>
+      <c r="H33" s="100"/>
+      <c r="I33" s="100"/>
+      <c r="J33" s="100"/>
       <c r="K33" s="47"/>
       <c r="L33" s="48"/>
       <c r="M33" s="49"/>
@@ -4130,20 +4139,20 @@
       <c r="V33" s="49"/>
       <c r="W33" s="47"/>
       <c r="X33" s="50"/>
-      <c r="Y33" s="159">
+      <c r="Y33" s="101">
         <v>15</v>
       </c>
-      <c r="Z33" s="154"/>
-      <c r="AA33" s="167"/>
-      <c r="AB33" s="167"/>
-      <c r="AC33" s="167"/>
-      <c r="AD33" s="167"/>
-      <c r="AE33" s="167"/>
-      <c r="AF33" s="161"/>
-      <c r="AG33" s="161"/>
-      <c r="AH33" s="161"/>
-      <c r="AI33" s="162"/>
-      <c r="AJ33" s="163"/>
+      <c r="Z33" s="96"/>
+      <c r="AA33" s="105"/>
+      <c r="AB33" s="105"/>
+      <c r="AC33" s="105"/>
+      <c r="AD33" s="105"/>
+      <c r="AE33" s="105"/>
+      <c r="AF33" s="106"/>
+      <c r="AG33" s="106"/>
+      <c r="AH33" s="106"/>
+      <c r="AI33" s="93"/>
+      <c r="AJ33" s="94"/>
       <c r="AK33" s="49"/>
       <c r="AL33" s="47"/>
       <c r="AM33" s="48"/>
@@ -4158,18 +4167,18 @@
       <c r="AV33" s="51"/>
     </row>
     <row r="34" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A34" s="153">
+      <c r="A34" s="95">
         <v>5</v>
       </c>
-      <c r="B34" s="154"/>
-      <c r="C34" s="155"/>
-      <c r="D34" s="156"/>
-      <c r="E34" s="156"/>
-      <c r="F34" s="156"/>
-      <c r="G34" s="157"/>
-      <c r="H34" s="158"/>
-      <c r="I34" s="158"/>
-      <c r="J34" s="158"/>
+      <c r="B34" s="96"/>
+      <c r="C34" s="97"/>
+      <c r="D34" s="98"/>
+      <c r="E34" s="98"/>
+      <c r="F34" s="98"/>
+      <c r="G34" s="99"/>
+      <c r="H34" s="100"/>
+      <c r="I34" s="100"/>
+      <c r="J34" s="100"/>
       <c r="K34" s="47"/>
       <c r="L34" s="48"/>
       <c r="M34" s="49"/>
@@ -4184,20 +4193,20 @@
       <c r="V34" s="49"/>
       <c r="W34" s="47"/>
       <c r="X34" s="50"/>
-      <c r="Y34" s="159">
+      <c r="Y34" s="101">
         <v>16</v>
       </c>
-      <c r="Z34" s="154"/>
-      <c r="AA34" s="169"/>
-      <c r="AB34" s="169"/>
-      <c r="AC34" s="169"/>
-      <c r="AD34" s="169"/>
-      <c r="AE34" s="169"/>
-      <c r="AF34" s="170"/>
-      <c r="AG34" s="170"/>
-      <c r="AH34" s="170"/>
-      <c r="AI34" s="162"/>
-      <c r="AJ34" s="163"/>
+      <c r="Z34" s="96"/>
+      <c r="AA34" s="102"/>
+      <c r="AB34" s="102"/>
+      <c r="AC34" s="102"/>
+      <c r="AD34" s="102"/>
+      <c r="AE34" s="102"/>
+      <c r="AF34" s="103"/>
+      <c r="AG34" s="103"/>
+      <c r="AH34" s="103"/>
+      <c r="AI34" s="93"/>
+      <c r="AJ34" s="94"/>
       <c r="AK34" s="49"/>
       <c r="AL34" s="47"/>
       <c r="AM34" s="48"/>
@@ -4212,18 +4221,18 @@
       <c r="AV34" s="51"/>
     </row>
     <row r="35" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A35" s="153">
+      <c r="A35" s="95">
         <v>6</v>
       </c>
-      <c r="B35" s="154"/>
-      <c r="C35" s="155"/>
-      <c r="D35" s="156"/>
-      <c r="E35" s="156"/>
-      <c r="F35" s="156"/>
-      <c r="G35" s="157"/>
-      <c r="H35" s="158"/>
-      <c r="I35" s="158"/>
-      <c r="J35" s="158"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="97"/>
+      <c r="D35" s="98"/>
+      <c r="E35" s="98"/>
+      <c r="F35" s="98"/>
+      <c r="G35" s="99"/>
+      <c r="H35" s="100"/>
+      <c r="I35" s="100"/>
+      <c r="J35" s="100"/>
       <c r="K35" s="47"/>
       <c r="L35" s="48"/>
       <c r="M35" s="49"/>
@@ -4238,20 +4247,20 @@
       <c r="V35" s="49"/>
       <c r="W35" s="47"/>
       <c r="X35" s="50"/>
-      <c r="Y35" s="159">
+      <c r="Y35" s="101">
         <v>17</v>
       </c>
-      <c r="Z35" s="154"/>
-      <c r="AA35" s="169"/>
-      <c r="AB35" s="169"/>
-      <c r="AC35" s="169"/>
-      <c r="AD35" s="169"/>
-      <c r="AE35" s="169"/>
-      <c r="AF35" s="170"/>
-      <c r="AG35" s="170"/>
-      <c r="AH35" s="170"/>
-      <c r="AI35" s="162"/>
-      <c r="AJ35" s="163"/>
+      <c r="Z35" s="96"/>
+      <c r="AA35" s="102"/>
+      <c r="AB35" s="102"/>
+      <c r="AC35" s="102"/>
+      <c r="AD35" s="102"/>
+      <c r="AE35" s="102"/>
+      <c r="AF35" s="103"/>
+      <c r="AG35" s="103"/>
+      <c r="AH35" s="103"/>
+      <c r="AI35" s="93"/>
+      <c r="AJ35" s="94"/>
       <c r="AK35" s="49"/>
       <c r="AL35" s="47"/>
       <c r="AM35" s="48"/>
@@ -4266,18 +4275,18 @@
       <c r="AV35" s="51"/>
     </row>
     <row r="36" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A36" s="153">
+      <c r="A36" s="95">
         <v>7</v>
       </c>
-      <c r="B36" s="154"/>
-      <c r="C36" s="155"/>
-      <c r="D36" s="156"/>
-      <c r="E36" s="156"/>
-      <c r="F36" s="156"/>
-      <c r="G36" s="157"/>
-      <c r="H36" s="171"/>
-      <c r="I36" s="171"/>
-      <c r="J36" s="171"/>
+      <c r="B36" s="96"/>
+      <c r="C36" s="97"/>
+      <c r="D36" s="98"/>
+      <c r="E36" s="98"/>
+      <c r="F36" s="98"/>
+      <c r="G36" s="99"/>
+      <c r="H36" s="104"/>
+      <c r="I36" s="104"/>
+      <c r="J36" s="104"/>
       <c r="K36" s="47"/>
       <c r="L36" s="48"/>
       <c r="M36" s="49"/>
@@ -4292,20 +4301,20 @@
       <c r="V36" s="49"/>
       <c r="W36" s="47"/>
       <c r="X36" s="50"/>
-      <c r="Y36" s="159">
+      <c r="Y36" s="101">
         <v>18</v>
       </c>
-      <c r="Z36" s="154"/>
-      <c r="AA36" s="169"/>
-      <c r="AB36" s="169"/>
-      <c r="AC36" s="169"/>
-      <c r="AD36" s="169"/>
-      <c r="AE36" s="169"/>
-      <c r="AF36" s="170"/>
-      <c r="AG36" s="170"/>
-      <c r="AH36" s="170"/>
-      <c r="AI36" s="162"/>
-      <c r="AJ36" s="163"/>
+      <c r="Z36" s="96"/>
+      <c r="AA36" s="102"/>
+      <c r="AB36" s="102"/>
+      <c r="AC36" s="102"/>
+      <c r="AD36" s="102"/>
+      <c r="AE36" s="102"/>
+      <c r="AF36" s="103"/>
+      <c r="AG36" s="103"/>
+      <c r="AH36" s="103"/>
+      <c r="AI36" s="93"/>
+      <c r="AJ36" s="94"/>
       <c r="AK36" s="49"/>
       <c r="AL36" s="47"/>
       <c r="AM36" s="48"/>
@@ -4320,18 +4329,18 @@
       <c r="AV36" s="51"/>
     </row>
     <row r="37" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A37" s="153">
+      <c r="A37" s="95">
         <v>8</v>
       </c>
-      <c r="B37" s="154"/>
-      <c r="C37" s="155"/>
-      <c r="D37" s="156"/>
-      <c r="E37" s="156"/>
-      <c r="F37" s="156"/>
-      <c r="G37" s="157"/>
-      <c r="H37" s="158"/>
-      <c r="I37" s="158"/>
-      <c r="J37" s="158"/>
+      <c r="B37" s="96"/>
+      <c r="C37" s="97"/>
+      <c r="D37" s="98"/>
+      <c r="E37" s="98"/>
+      <c r="F37" s="98"/>
+      <c r="G37" s="99"/>
+      <c r="H37" s="100"/>
+      <c r="I37" s="100"/>
+      <c r="J37" s="100"/>
       <c r="K37" s="47"/>
       <c r="L37" s="48"/>
       <c r="M37" s="49"/>
@@ -4346,20 +4355,20 @@
       <c r="V37" s="49"/>
       <c r="W37" s="47"/>
       <c r="X37" s="50"/>
-      <c r="Y37" s="159">
+      <c r="Y37" s="101">
         <v>19</v>
       </c>
-      <c r="Z37" s="154"/>
-      <c r="AA37" s="169"/>
-      <c r="AB37" s="169"/>
-      <c r="AC37" s="169"/>
-      <c r="AD37" s="169"/>
-      <c r="AE37" s="169"/>
-      <c r="AF37" s="170"/>
-      <c r="AG37" s="170"/>
-      <c r="AH37" s="170"/>
-      <c r="AI37" s="162"/>
-      <c r="AJ37" s="163"/>
+      <c r="Z37" s="96"/>
+      <c r="AA37" s="102"/>
+      <c r="AB37" s="102"/>
+      <c r="AC37" s="102"/>
+      <c r="AD37" s="102"/>
+      <c r="AE37" s="102"/>
+      <c r="AF37" s="103"/>
+      <c r="AG37" s="103"/>
+      <c r="AH37" s="103"/>
+      <c r="AI37" s="93"/>
+      <c r="AJ37" s="94"/>
       <c r="AK37" s="49"/>
       <c r="AL37" s="47"/>
       <c r="AM37" s="48"/>
@@ -4374,18 +4383,18 @@
       <c r="AV37" s="51"/>
     </row>
     <row r="38" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A38" s="153">
+      <c r="A38" s="95">
         <v>9</v>
       </c>
-      <c r="B38" s="154"/>
-      <c r="C38" s="155"/>
-      <c r="D38" s="156"/>
-      <c r="E38" s="156"/>
-      <c r="F38" s="156"/>
-      <c r="G38" s="157"/>
-      <c r="H38" s="158"/>
-      <c r="I38" s="158"/>
-      <c r="J38" s="158"/>
+      <c r="B38" s="96"/>
+      <c r="C38" s="97"/>
+      <c r="D38" s="98"/>
+      <c r="E38" s="98"/>
+      <c r="F38" s="98"/>
+      <c r="G38" s="99"/>
+      <c r="H38" s="100"/>
+      <c r="I38" s="100"/>
+      <c r="J38" s="100"/>
       <c r="K38" s="47"/>
       <c r="L38" s="48"/>
       <c r="M38" s="49"/>
@@ -4400,20 +4409,20 @@
       <c r="V38" s="49"/>
       <c r="W38" s="47"/>
       <c r="X38" s="50"/>
-      <c r="Y38" s="159">
+      <c r="Y38" s="101">
         <v>20</v>
       </c>
-      <c r="Z38" s="154"/>
-      <c r="AA38" s="169"/>
-      <c r="AB38" s="169"/>
-      <c r="AC38" s="169"/>
-      <c r="AD38" s="169"/>
-      <c r="AE38" s="169"/>
-      <c r="AF38" s="170"/>
-      <c r="AG38" s="170"/>
-      <c r="AH38" s="170"/>
-      <c r="AI38" s="162"/>
-      <c r="AJ38" s="163"/>
+      <c r="Z38" s="96"/>
+      <c r="AA38" s="102"/>
+      <c r="AB38" s="102"/>
+      <c r="AC38" s="102"/>
+      <c r="AD38" s="102"/>
+      <c r="AE38" s="102"/>
+      <c r="AF38" s="103"/>
+      <c r="AG38" s="103"/>
+      <c r="AH38" s="103"/>
+      <c r="AI38" s="93"/>
+      <c r="AJ38" s="94"/>
       <c r="AK38" s="49"/>
       <c r="AL38" s="47"/>
       <c r="AM38" s="48"/>
@@ -4428,18 +4437,18 @@
       <c r="AV38" s="51"/>
     </row>
     <row r="39" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A39" s="153">
+      <c r="A39" s="95">
         <v>10</v>
       </c>
-      <c r="B39" s="154"/>
-      <c r="C39" s="155"/>
-      <c r="D39" s="156"/>
-      <c r="E39" s="156"/>
-      <c r="F39" s="156"/>
-      <c r="G39" s="157"/>
-      <c r="H39" s="158"/>
-      <c r="I39" s="158"/>
-      <c r="J39" s="158"/>
+      <c r="B39" s="96"/>
+      <c r="C39" s="97"/>
+      <c r="D39" s="98"/>
+      <c r="E39" s="98"/>
+      <c r="F39" s="98"/>
+      <c r="G39" s="99"/>
+      <c r="H39" s="100"/>
+      <c r="I39" s="100"/>
+      <c r="J39" s="100"/>
       <c r="K39" s="47"/>
       <c r="L39" s="48"/>
       <c r="M39" s="49"/>
@@ -4454,20 +4463,20 @@
       <c r="V39" s="49"/>
       <c r="W39" s="47"/>
       <c r="X39" s="50"/>
-      <c r="Y39" s="159">
+      <c r="Y39" s="101">
         <v>21</v>
       </c>
-      <c r="Z39" s="154"/>
-      <c r="AA39" s="169"/>
-      <c r="AB39" s="169"/>
-      <c r="AC39" s="169"/>
-      <c r="AD39" s="169"/>
-      <c r="AE39" s="169"/>
-      <c r="AF39" s="170"/>
-      <c r="AG39" s="170"/>
-      <c r="AH39" s="170"/>
-      <c r="AI39" s="162"/>
-      <c r="AJ39" s="163"/>
+      <c r="Z39" s="96"/>
+      <c r="AA39" s="102"/>
+      <c r="AB39" s="102"/>
+      <c r="AC39" s="102"/>
+      <c r="AD39" s="102"/>
+      <c r="AE39" s="102"/>
+      <c r="AF39" s="103"/>
+      <c r="AG39" s="103"/>
+      <c r="AH39" s="103"/>
+      <c r="AI39" s="93"/>
+      <c r="AJ39" s="94"/>
       <c r="AK39" s="49"/>
       <c r="AL39" s="47"/>
       <c r="AM39" s="48"/>
@@ -4482,18 +4491,18 @@
       <c r="AV39" s="51"/>
     </row>
     <row r="40" spans="1:48" s="13" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A40" s="153">
+      <c r="A40" s="95">
         <v>11</v>
       </c>
-      <c r="B40" s="154"/>
-      <c r="C40" s="155"/>
-      <c r="D40" s="156"/>
-      <c r="E40" s="156"/>
-      <c r="F40" s="156"/>
-      <c r="G40" s="157"/>
-      <c r="H40" s="158"/>
-      <c r="I40" s="158"/>
-      <c r="J40" s="158"/>
+      <c r="B40" s="96"/>
+      <c r="C40" s="97"/>
+      <c r="D40" s="98"/>
+      <c r="E40" s="98"/>
+      <c r="F40" s="98"/>
+      <c r="G40" s="99"/>
+      <c r="H40" s="100"/>
+      <c r="I40" s="100"/>
+      <c r="J40" s="100"/>
       <c r="K40" s="47"/>
       <c r="L40" s="48"/>
       <c r="M40" s="49"/>
@@ -4508,20 +4517,20 @@
       <c r="V40" s="49"/>
       <c r="W40" s="47"/>
       <c r="X40" s="50"/>
-      <c r="Y40" s="159">
+      <c r="Y40" s="101">
         <v>22</v>
       </c>
-      <c r="Z40" s="154"/>
-      <c r="AA40" s="169"/>
-      <c r="AB40" s="169"/>
-      <c r="AC40" s="169"/>
-      <c r="AD40" s="169"/>
-      <c r="AE40" s="169"/>
-      <c r="AF40" s="170"/>
-      <c r="AG40" s="170"/>
-      <c r="AH40" s="170"/>
-      <c r="AI40" s="162"/>
-      <c r="AJ40" s="163"/>
+      <c r="Z40" s="96"/>
+      <c r="AA40" s="102"/>
+      <c r="AB40" s="102"/>
+      <c r="AC40" s="102"/>
+      <c r="AD40" s="102"/>
+      <c r="AE40" s="102"/>
+      <c r="AF40" s="103"/>
+      <c r="AG40" s="103"/>
+      <c r="AH40" s="103"/>
+      <c r="AI40" s="93"/>
+      <c r="AJ40" s="94"/>
       <c r="AK40" s="49"/>
       <c r="AL40" s="47"/>
       <c r="AM40" s="48"/>
@@ -4536,18 +4545,18 @@
       <c r="AV40" s="51"/>
     </row>
     <row r="41" spans="1:48" s="13" customFormat="1" ht="20.25" customHeight="1" thickBot="1">
-      <c r="A41" s="174" t="s">
+      <c r="A41" s="83" t="s">
         <v>69</v>
       </c>
-      <c r="B41" s="175"/>
-      <c r="C41" s="175"/>
-      <c r="D41" s="175"/>
-      <c r="E41" s="175"/>
-      <c r="F41" s="175"/>
-      <c r="G41" s="175"/>
-      <c r="H41" s="175"/>
-      <c r="I41" s="175"/>
-      <c r="J41" s="175"/>
+      <c r="B41" s="84"/>
+      <c r="C41" s="84"/>
+      <c r="D41" s="84"/>
+      <c r="E41" s="84"/>
+      <c r="F41" s="84"/>
+      <c r="G41" s="84"/>
+      <c r="H41" s="84"/>
+      <c r="I41" s="84"/>
+      <c r="J41" s="84"/>
       <c r="K41" s="52"/>
       <c r="L41" s="53"/>
       <c r="M41" s="52"/>
@@ -4562,20 +4571,20 @@
       <c r="V41" s="56"/>
       <c r="W41" s="54"/>
       <c r="X41" s="57"/>
-      <c r="Y41" s="176" t="s">
+      <c r="Y41" s="85" t="s">
         <v>69</v>
       </c>
-      <c r="Z41" s="177"/>
-      <c r="AA41" s="177"/>
-      <c r="AB41" s="177"/>
-      <c r="AC41" s="177"/>
-      <c r="AD41" s="177"/>
-      <c r="AE41" s="177"/>
-      <c r="AF41" s="177"/>
-      <c r="AG41" s="177"/>
-      <c r="AH41" s="178"/>
-      <c r="AI41" s="179"/>
-      <c r="AJ41" s="178"/>
+      <c r="Z41" s="86"/>
+      <c r="AA41" s="86"/>
+      <c r="AB41" s="86"/>
+      <c r="AC41" s="86"/>
+      <c r="AD41" s="86"/>
+      <c r="AE41" s="86"/>
+      <c r="AF41" s="86"/>
+      <c r="AG41" s="86"/>
+      <c r="AH41" s="87"/>
+      <c r="AI41" s="88"/>
+      <c r="AJ41" s="87"/>
       <c r="AK41" s="52"/>
       <c r="AL41" s="58"/>
       <c r="AM41" s="53"/>
@@ -4613,31 +4622,31 @@
       <c r="V42" s="61"/>
       <c r="W42" s="61"/>
       <c r="X42" s="61"/>
-      <c r="AD42" s="180" t="s">
+      <c r="AD42" s="89" t="s">
         <v>71</v>
       </c>
-      <c r="AE42" s="180"/>
-      <c r="AF42" s="180"/>
-      <c r="AG42" s="180"/>
-      <c r="AH42" s="180"/>
-      <c r="AI42" s="180"/>
-      <c r="AJ42" s="180"/>
-      <c r="AK42" s="94" t="s">
+      <c r="AE42" s="89"/>
+      <c r="AF42" s="89"/>
+      <c r="AG42" s="89"/>
+      <c r="AH42" s="89"/>
+      <c r="AI42" s="89"/>
+      <c r="AJ42" s="89"/>
+      <c r="AK42" s="90" t="s">
         <v>72</v>
       </c>
-      <c r="AL42" s="94"/>
-      <c r="AM42" s="94"/>
-      <c r="AN42" s="94"/>
-      <c r="AO42" s="94"/>
-      <c r="AP42" s="94"/>
-      <c r="AQ42" s="93" t="s">
+      <c r="AL42" s="90"/>
+      <c r="AM42" s="90"/>
+      <c r="AN42" s="90"/>
+      <c r="AO42" s="90"/>
+      <c r="AP42" s="90"/>
+      <c r="AQ42" s="91" t="s">
         <v>73</v>
       </c>
-      <c r="AR42" s="94"/>
-      <c r="AS42" s="94"/>
-      <c r="AT42" s="94"/>
-      <c r="AU42" s="94"/>
-      <c r="AV42" s="98"/>
+      <c r="AR42" s="90"/>
+      <c r="AS42" s="90"/>
+      <c r="AT42" s="90"/>
+      <c r="AU42" s="90"/>
+      <c r="AV42" s="92"/>
     </row>
     <row r="43" spans="1:48" s="13" customFormat="1" ht="36" customHeight="1" thickBot="1">
       <c r="A43" s="62"/>
@@ -4669,25 +4678,25 @@
       <c r="AA43" s="63"/>
       <c r="AB43" s="63"/>
       <c r="AC43" s="63"/>
-      <c r="AD43" s="172"/>
-      <c r="AE43" s="172"/>
-      <c r="AF43" s="172"/>
-      <c r="AG43" s="172"/>
-      <c r="AH43" s="172"/>
-      <c r="AI43" s="172"/>
-      <c r="AJ43" s="172"/>
-      <c r="AK43" s="172"/>
-      <c r="AL43" s="172"/>
-      <c r="AM43" s="172"/>
-      <c r="AN43" s="172"/>
-      <c r="AO43" s="172"/>
-      <c r="AP43" s="172"/>
-      <c r="AQ43" s="172"/>
-      <c r="AR43" s="172"/>
-      <c r="AS43" s="172"/>
-      <c r="AT43" s="172"/>
-      <c r="AU43" s="172"/>
-      <c r="AV43" s="173"/>
+      <c r="AD43" s="81"/>
+      <c r="AE43" s="81"/>
+      <c r="AF43" s="81"/>
+      <c r="AG43" s="81"/>
+      <c r="AH43" s="81"/>
+      <c r="AI43" s="81"/>
+      <c r="AJ43" s="81"/>
+      <c r="AK43" s="81"/>
+      <c r="AL43" s="81"/>
+      <c r="AM43" s="81"/>
+      <c r="AN43" s="81"/>
+      <c r="AO43" s="81"/>
+      <c r="AP43" s="81"/>
+      <c r="AQ43" s="81"/>
+      <c r="AR43" s="81"/>
+      <c r="AS43" s="81"/>
+      <c r="AT43" s="81"/>
+      <c r="AU43" s="81"/>
+      <c r="AV43" s="82"/>
     </row>
     <row r="44" spans="1:48" s="13" customFormat="1" ht="12.75"/>
     <row r="45" spans="1:48" s="13" customFormat="1" ht="12.75"/>
@@ -4701,85 +4710,46 @@
     <row r="53" s="13" customFormat="1" ht="12.75"/>
   </sheetData>
   <mergeCells count="137">
-    <mergeCell ref="AD43:AJ43"/>
-    <mergeCell ref="AK43:AP43"/>
-    <mergeCell ref="AQ43:AV43"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="Y41:AH41"/>
-    <mergeCell ref="AI41:AJ41"/>
-    <mergeCell ref="AD42:AJ42"/>
-    <mergeCell ref="AK42:AP42"/>
-    <mergeCell ref="AQ42:AV42"/>
-    <mergeCell ref="AI39:AJ39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="Y40:Z40"/>
-    <mergeCell ref="AA40:AE40"/>
-    <mergeCell ref="AF40:AH40"/>
-    <mergeCell ref="AI40:AJ40"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="Y39:Z39"/>
-    <mergeCell ref="AA39:AE39"/>
-    <mergeCell ref="AF39:AH39"/>
-    <mergeCell ref="AI37:AJ37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="Y38:Z38"/>
-    <mergeCell ref="AA38:AE38"/>
-    <mergeCell ref="AF38:AH38"/>
-    <mergeCell ref="AI38:AJ38"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="H37:J37"/>
-    <mergeCell ref="Y37:Z37"/>
-    <mergeCell ref="AA37:AE37"/>
-    <mergeCell ref="AF37:AH37"/>
-    <mergeCell ref="AI35:AJ35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="Y36:Z36"/>
-    <mergeCell ref="AA36:AE36"/>
-    <mergeCell ref="AF36:AH36"/>
-    <mergeCell ref="AI36:AJ36"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="Y35:Z35"/>
-    <mergeCell ref="AA35:AE35"/>
-    <mergeCell ref="AF35:AH35"/>
-    <mergeCell ref="AI33:AJ33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="AA34:AE34"/>
-    <mergeCell ref="AF34:AH34"/>
-    <mergeCell ref="AI34:AJ34"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="H33:J33"/>
-    <mergeCell ref="Y33:Z33"/>
-    <mergeCell ref="AA33:AE33"/>
-    <mergeCell ref="AF33:AH33"/>
-    <mergeCell ref="AI31:AJ31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="Y32:Z32"/>
-    <mergeCell ref="AA32:AE32"/>
-    <mergeCell ref="AF32:AH32"/>
-    <mergeCell ref="AI32:AJ32"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="Y31:Z31"/>
-    <mergeCell ref="AA31:AE31"/>
-    <mergeCell ref="AF31:AH31"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="I6:T6"/>
+    <mergeCell ref="U6:AA6"/>
+    <mergeCell ref="AB6:AH6"/>
+    <mergeCell ref="AI6:AO6"/>
+    <mergeCell ref="AP6:AV6"/>
+    <mergeCell ref="O2:AM3"/>
+    <mergeCell ref="AO3:AS3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="I5:T5"/>
+    <mergeCell ref="U5:AA5"/>
+    <mergeCell ref="AB5:AH5"/>
+    <mergeCell ref="AI5:AO5"/>
+    <mergeCell ref="AP5:AV5"/>
+    <mergeCell ref="AC8:AE8"/>
+    <mergeCell ref="AG8:AS8"/>
+    <mergeCell ref="AT8:AV8"/>
+    <mergeCell ref="AC9:AE12"/>
+    <mergeCell ref="AC13:AE17"/>
+    <mergeCell ref="AG16:AS16"/>
+    <mergeCell ref="AT17:AV18"/>
+    <mergeCell ref="AC18:AE22"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="I7:T7"/>
+    <mergeCell ref="U7:AA7"/>
+    <mergeCell ref="AB7:AH7"/>
+    <mergeCell ref="AI7:AO7"/>
+    <mergeCell ref="AP7:AV7"/>
+    <mergeCell ref="AC23:AE26"/>
+    <mergeCell ref="AG23:AS23"/>
+    <mergeCell ref="AG24:AS24"/>
+    <mergeCell ref="AG25:AS25"/>
+    <mergeCell ref="AG26:AS26"/>
+    <mergeCell ref="A28:B29"/>
+    <mergeCell ref="C28:G29"/>
+    <mergeCell ref="H28:J29"/>
+    <mergeCell ref="K28:X28"/>
+    <mergeCell ref="Y28:Z29"/>
+    <mergeCell ref="AN29:AP29"/>
+    <mergeCell ref="AQ29:AS29"/>
     <mergeCell ref="AT29:AV29"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="C30:G30"/>
@@ -4798,51 +4768,90 @@
     <mergeCell ref="V29:X29"/>
     <mergeCell ref="AI29:AJ29"/>
     <mergeCell ref="AK29:AM29"/>
-    <mergeCell ref="AC23:AE26"/>
-    <mergeCell ref="AG23:AS23"/>
-    <mergeCell ref="AG24:AS24"/>
-    <mergeCell ref="AG25:AS25"/>
-    <mergeCell ref="AG26:AS26"/>
-    <mergeCell ref="A28:B29"/>
-    <mergeCell ref="C28:G29"/>
-    <mergeCell ref="H28:J29"/>
-    <mergeCell ref="K28:X28"/>
-    <mergeCell ref="Y28:Z29"/>
-    <mergeCell ref="AN29:AP29"/>
-    <mergeCell ref="AQ29:AS29"/>
-    <mergeCell ref="AC8:AE8"/>
-    <mergeCell ref="AG8:AS8"/>
-    <mergeCell ref="AT8:AV8"/>
-    <mergeCell ref="AC9:AE12"/>
-    <mergeCell ref="AC13:AE17"/>
-    <mergeCell ref="AG16:AS16"/>
-    <mergeCell ref="AT17:AV18"/>
-    <mergeCell ref="AC18:AE22"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="I7:T7"/>
-    <mergeCell ref="U7:AA7"/>
-    <mergeCell ref="AB7:AH7"/>
-    <mergeCell ref="AI7:AO7"/>
-    <mergeCell ref="AP7:AV7"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="I6:T6"/>
-    <mergeCell ref="U6:AA6"/>
-    <mergeCell ref="AB6:AH6"/>
-    <mergeCell ref="AI6:AO6"/>
-    <mergeCell ref="AP6:AV6"/>
-    <mergeCell ref="O2:AM3"/>
-    <mergeCell ref="AO3:AS3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="I5:T5"/>
-    <mergeCell ref="U5:AA5"/>
-    <mergeCell ref="AB5:AH5"/>
-    <mergeCell ref="AI5:AO5"/>
-    <mergeCell ref="AP5:AV5"/>
+    <mergeCell ref="AI31:AJ31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="Y32:Z32"/>
+    <mergeCell ref="AA32:AE32"/>
+    <mergeCell ref="AF32:AH32"/>
+    <mergeCell ref="AI32:AJ32"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="Y31:Z31"/>
+    <mergeCell ref="AA31:AE31"/>
+    <mergeCell ref="AF31:AH31"/>
+    <mergeCell ref="AI33:AJ33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="AA34:AE34"/>
+    <mergeCell ref="AF34:AH34"/>
+    <mergeCell ref="AI34:AJ34"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="H33:J33"/>
+    <mergeCell ref="Y33:Z33"/>
+    <mergeCell ref="AA33:AE33"/>
+    <mergeCell ref="AF33:AH33"/>
+    <mergeCell ref="AI35:AJ35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="Y36:Z36"/>
+    <mergeCell ref="AA36:AE36"/>
+    <mergeCell ref="AF36:AH36"/>
+    <mergeCell ref="AI36:AJ36"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="Y35:Z35"/>
+    <mergeCell ref="AA35:AE35"/>
+    <mergeCell ref="AF35:AH35"/>
+    <mergeCell ref="AI37:AJ37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="Y38:Z38"/>
+    <mergeCell ref="AA38:AE38"/>
+    <mergeCell ref="AF38:AH38"/>
+    <mergeCell ref="AI38:AJ38"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="Y37:Z37"/>
+    <mergeCell ref="AA37:AE37"/>
+    <mergeCell ref="AF37:AH37"/>
+    <mergeCell ref="AI39:AJ39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="Y40:Z40"/>
+    <mergeCell ref="AA40:AE40"/>
+    <mergeCell ref="AF40:AH40"/>
+    <mergeCell ref="AI40:AJ40"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="Y39:Z39"/>
+    <mergeCell ref="AA39:AE39"/>
+    <mergeCell ref="AF39:AH39"/>
+    <mergeCell ref="AD43:AJ43"/>
+    <mergeCell ref="AK43:AP43"/>
+    <mergeCell ref="AQ43:AV43"/>
+    <mergeCell ref="A41:J41"/>
+    <mergeCell ref="Y41:AH41"/>
+    <mergeCell ref="AI41:AJ41"/>
+    <mergeCell ref="AD42:AJ42"/>
+    <mergeCell ref="AK42:AP42"/>
+    <mergeCell ref="AQ42:AV42"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="83" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rIdTextBoxes"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revise template and add button delete record
</commit_message>
<xml_diff>
--- a/templates/Spec.xlsx
+++ b/templates/Spec.xlsx
@@ -1973,16 +1973,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
+      <xdr:rowOff>266700</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2023,15 +2023,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>200025</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2071,16 +2071,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
+      <xdr:col>28</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>295275</xdr:rowOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2120,16 +2120,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>266700</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2163,6 +2163,216 @@
           <a:tailEnd type="none" w="med" len="med"/>
         </a:ln>
         <a:effectLst/>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="100" name="WireResultLine" hidden="1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="101" name="TerminalResultLine" hidden="1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="102" name="HousingResultLine" hidden="1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="103" name="OtherResultLine" hidden="1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="104" name="LengthLine1" hidden="1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>48</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="105" name="LengthLine2" hidden="1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
       </xdr:spPr>
     </xdr:cxnSp>
     <xdr:clientData/>

</xml_diff>